<commit_message>
feat(data): aggiorna rete geospaziale a Snapshot 3 (63 feature, 21.72 km)
- sposta i KML storici e il nuovo rilievo in data/snapshots/ (snapshot 1, 2, 3)
- redige data/snapshots/CHANGELOG_DATI.md con differenze e metriche storiche
- aggiorna scripts/kml_to_geojson.py per Snapshot 3 (nuove categorie e toponimi)
- aggiorna scripts/export_sheets.py con etichette coerenti e stato cantieri non collegati
- rigenera network_data.json, js/data.js, CSV e XLSX: 63 feature, 21.716 km totali
- +14 feature: Cantiere 3 Via Aiaccia (+3.48 km), INFRATEL 2 (+3.46 km), posa Stagno (+0.83 km),
  opera backbone (+0.52 km), armadi S [03] ARL, S [27] ARLO, S [28] ARLO, centrale feeder Livorno
- aggiornamento cantieri: C1 suddiviso in tratti eseguiti/non eseguiti, C2 slittato al 05/10
</commit_message>
<xml_diff>
--- a/data/rete_ftth_collesalvetti.xlsx
+++ b/data/rete_ftth_collesalvetti.xlsx
@@ -160,12 +160,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -180,7 +180,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>NON_ESEGUITO</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -205,14 +205,14 @@
         <v>10.473372</v>
       </c>
       <c r="M2">
-        <v>1096.2</v>
+        <v>384.6</v>
       </c>
       <c r="N2">
-        <v>1.096</v>
+        <v>0.385</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -234,12 +234,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 ESEGUITO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Eseguita)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -254,7 +254,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>ESEGUITO</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -273,25 +273,25 @@
         </is>
       </c>
       <c r="J3">
-        <v>43.595559</v>
+        <v>43.597359</v>
       </c>
       <c r="K3">
-        <v>10.477378</v>
+        <v>10.478268</v>
       </c>
       <c r="M3">
-        <v>325.2</v>
+        <v>580.3</v>
       </c>
       <c r="N3">
-        <v>0.325</v>
+        <v>0.58</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Tratta stabilita con un walk-in in data 29/09/2026 e 03/10/2026. Si notano minitrincee, matasse di corrugati e birilli. Oltre a una serie di pozzetti Fibercop.</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=43.595559,10.477378</t>
+          <t>https://www.google.com/maps?q=43.597359,10.478268</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>S [0?] ARLO</t>
+          <t>S [28] ARLO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1598,6 +1598,11 @@
       <c r="L32">
         <v>0.0</v>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Frazione di Parrana San Martino</t>
+        </is>
+      </c>
       <c r="R32" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.538167,10.442333</t>
@@ -1639,6 +1644,11 @@
       <c r="L33">
         <v>0.0</v>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Frazione di Parrana San Giusto</t>
+        </is>
+      </c>
       <c r="R33" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.528528,10.457333</t>
@@ -1831,12 +1841,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1851,7 +1861,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>NON_ESEGUITO</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1883,7 +1893,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -1905,12 +1915,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1925,7 +1935,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>NON_ESEGUITO</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1957,7 +1967,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -1979,12 +1989,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 ESEGUITO</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Eseguita)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1999,7 +2009,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>ESEGUITO</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2018,25 +2028,25 @@
         </is>
       </c>
       <c r="J40">
-        <v>43.593821</v>
+        <v>43.595583</v>
       </c>
       <c r="K40">
-        <v>10.475403</v>
+        <v>10.474905</v>
       </c>
       <c r="M40">
-        <v>293.4</v>
+        <v>496.3</v>
       </c>
       <c r="N40">
-        <v>0.293</v>
+        <v>0.496</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Tratta stabilita con un walk-in in data 29/09/2026 e 03/10/2026. Si notano minitrincee, matasse di corrugati e birilli. Oltre a una serie di pozzetti Fibercop.</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=43.593821,10.475403</t>
+          <t>https://www.google.com/maps?q=43.595583,10.474905</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -2053,12 +2063,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cantiere 1 (14/09-02/10)</t>
+          <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Cantiere FTTH (Attivazione Imminente)</t>
+          <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2073,7 +2083,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>IMMINENTE</t>
+          <t>NON_ESEGUITO</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2105,7 +2115,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Cantiere FTTH FiberCop Collesalvetti (Ord. 95/2026 del 02/09/2026). Vie: Via Nenni, Via Roma, Via del Valico a Pisa, Via di Cerretello.</t>
+          <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -2127,7 +2137,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Area Coperta</t>
+          <t>Area Coperta Collesalvetti</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2137,7 +2147,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Altro</t>
+          <t>Collesalvetti</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2171,17 +2181,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>Area NON Coperta Collesalvetti</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>Area NON Coperta</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Area NON Coperta</t>
-        </is>
-      </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Altro</t>
+          <t>Collesalvetti</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2401,7 +2411,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cantiere 2 (21/09-16/10)</t>
+          <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2453,7 +2463,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Nuovo cantiere FTTH FiberCop Stagno (Ord. 102/2026 del 10/09/2026). Vie: Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio.</t>
+          <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -2475,7 +2485,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cantiere 2 (21/09-16/10)</t>
+          <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2527,7 +2537,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Nuovo cantiere FTTH FiberCop Stagno (Ord. 102/2026 del 10/09/2026). Vie: Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio.</t>
+          <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -2549,7 +2559,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cantiere 2 (21/09-16/10)</t>
+          <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2601,7 +2611,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Nuovo cantiere FTTH FiberCop Stagno (Ord. 102/2026 del 10/09/2026). Vie: Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio.</t>
+          <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -2612,6 +2622,688 @@
       <c r="S50" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_102_2026_stagno_cantiere2.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>05C7B1F97841C1CA147C</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Opera sulla Backbone di 07/2026</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dorsale / Backbone Fibra</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J51">
+        <v>43.571782</v>
+      </c>
+      <c r="K51">
+        <v>10.369152</v>
+      </c>
+      <c r="M51">
+        <v>519.2</v>
+      </c>
+      <c r="N51">
+        <v>0.519</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Opera di Fibercop su una tratta di backbone in fibra che va verso est quindi presumibilmente verso Collesalvetti. Ordinanza allegata...</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.571782,10.369152</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>05B932036B41C1D8F728</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>INFRATEL</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Infrastruttura Infratel BUL</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J52">
+        <v>43.538194</v>
+      </c>
+      <c r="K52">
+        <v>10.442316</v>
+      </c>
+      <c r="M52">
+        <v>3462.3</v>
+      </c>
+      <c r="N52">
+        <v>3.462</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Seconda ed ultima tratta di INFRATEL per rilegare le centrali di Parrana San Martino e Parrana San Giusto in fibra ottica. Prevalentemente in palifica (specialmente a nord-ovest)</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.538194,10.442316</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>0A2895209441C56CED8C</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>S [27] ARLO</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ARLO (Ottico FiberCop)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J53">
+        <v>43.592688</v>
+      </c>
+      <c r="K53">
+        <v>10.350454</v>
+      </c>
+      <c r="L53">
+        <v>2.5</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.592688,10.350454</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06D2B51C4A41C5796F90</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>S [03] ARL</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ARL (Rame)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J54">
+        <v>43.589284</v>
+      </c>
+      <c r="K54">
+        <v>10.355304</v>
+      </c>
+      <c r="L54">
+        <v>9.0</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Con apparato aggiuntivo</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.589284,10.355304</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>087416D75C41C59E4800</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Tratta Fibra Posa</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J55">
+        <v>43.59306</v>
+      </c>
+      <c r="K55">
+        <v>10.349492</v>
+      </c>
+      <c r="M55">
+        <v>250.1</v>
+      </c>
+      <c r="N55">
+        <v>0.25</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.59306,10.349492</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>023213B9C541C59EFAE8</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Tratta Fibra Posa</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J56">
+        <v>43.592858</v>
+      </c>
+      <c r="K56">
+        <v>10.350051</v>
+      </c>
+      <c r="M56">
+        <v>119.4</v>
+      </c>
+      <c r="N56">
+        <v>0.119</v>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.592858,10.350051</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>03B96D8A3141C59F56F7</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Tratta Fibra Posa</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J57">
+        <v>43.591477</v>
+      </c>
+      <c r="K57">
+        <v>10.349452</v>
+      </c>
+      <c r="M57">
+        <v>149.9</v>
+      </c>
+      <c r="N57">
+        <v>0.15</v>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.591477,10.349452</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>0AB38499FF41C59FB9EC</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Tratta Fibra Posa</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="J58">
+        <v>43.59114</v>
+      </c>
+      <c r="K58">
+        <v>10.350885</v>
+      </c>
+      <c r="M58">
+        <v>308.2</v>
+      </c>
+      <c r="N58">
+        <v>0.308</v>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.59114,10.350885</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>04A0FAC1A941E16312D8</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Centrale Feeder (Livorno Nord)</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Centrale Feeder (Interconnessione Esterna)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Altro</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="J59">
+        <v>43.549556</v>
+      </c>
+      <c r="K59">
+        <v>10.310667</v>
+      </c>
+      <c r="L59">
+        <v>0.0</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Grande centrale Fibercop che funge da "feeder" alla centrale comunale di Collesalvetti</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.549556,10.310667</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>0DE7916F26423746716E</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Cantiere 1 NON ESEGUITO</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Cantiere FTTH (Tratta Non Eseguita)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Collesalvetti</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>NON_ESEGUITO</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-09-14 -&gt; 2026-10-02</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
+        </is>
+      </c>
+      <c r="J60">
+        <v>43.595608</v>
+      </c>
+      <c r="K60">
+        <v>10.474975</v>
+      </c>
+      <c r="M60">
+        <v>182.8</v>
+      </c>
+      <c r="N60">
+        <v>0.183</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.595608,10.474975</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>0A173E317742376CD0E8</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Cantiere 3 (19/10-23/10)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Cantiere Fibra Ottica</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>DA COLLEGARE A ORDINANZA</t>
+        </is>
+      </c>
+      <c r="J61">
+        <v>43.581537</v>
+      </c>
+      <c r="K61">
+        <v>10.350735</v>
+      </c>
+      <c r="M61">
+        <v>172.7</v>
+      </c>
+      <c r="N61">
+        <v>0.173</v>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.581537,10.350735</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>0EB8D0BA5142376E2D37</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Cantiere 3 (19/10-23/10)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Cantiere Fibra Ottica</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>DA COLLEGARE A ORDINANZA</t>
+        </is>
+      </c>
+      <c r="J62">
+        <v>43.58171</v>
+      </c>
+      <c r="K62">
+        <v>10.343732</v>
+      </c>
+      <c r="M62">
+        <v>627.5</v>
+      </c>
+      <c r="N62">
+        <v>0.627</v>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.58171,10.343732</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>07624940EF4237721F0B</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Cantiere 3 (19/10-23/10)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Cantiere Fibra Ottica</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>DA COLLEGARE A ORDINANZA</t>
+        </is>
+      </c>
+      <c r="J63">
+        <v>43.581465</v>
+      </c>
+      <c r="K63">
+        <v>10.348597</v>
+      </c>
+      <c r="M63">
+        <v>2507.4</v>
+      </c>
+      <c r="N63">
+        <v>2.507</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Improbabile che il cantiere arrivi fino a queste zone, ma fino al 24 ottobre circa terrò sulla mappa tutta Via Aiaccia. Curioso che però questa tratta arriva davanti alla tratta color viola "Opera sulla Backbone di 07/26"... analisi di questa informazione è necessaria.</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.581465,10.348597</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>0C884334EF423778B430</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Cantiere 3 (19/10-23/10)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Cantiere Fibra Ottica</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>DA COLLEGARE A ORDINANZA</t>
+        </is>
+      </c>
+      <c r="J64">
+        <v>43.58522</v>
+      </c>
+      <c r="K64">
+        <v>10.353831</v>
+      </c>
+      <c r="M64">
+        <v>167.7</v>
+      </c>
+      <c r="N64">
+        <v>0.168</v>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.58522,10.353831</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(export): correggi escaping XML, aggiungi foglio INFO, freeze pane, autofilter e sanitizzazione
</commit_message>
<xml_diff>
--- a/data/rete_ftth_collesalvetti.xlsx
+++ b/data/rete_ftth_collesalvetti.xlsx
@@ -1,15 +1,21 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-    <sheets>
-        <sheet name="Rete FTTH & Cantieri" sheetId="1" r:id="rId1"/>
-    </sheets>
+  <sheets>
+    <sheet name="Rete FTTH &amp; Cantieri" sheetId="1" r:id="rId1"/>
+    <sheet name="INFO &amp; Metodologia" sheetId="2" r:id="rId2"/>
+  </sheets>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
@@ -20,8 +26,14 @@
       <b/>
       <color rgb="FFFFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+      <b/>
+      <color rgb="FF0F4C81"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -33,27 +45,68 @@
         <fgColor rgb="FF0F4C81"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF0F4F8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7DE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="9" max="9" width="45" customWidth="1"/>
+    <col min="10" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="13" max="14" width="16" customWidth="1"/>
+    <col min="15" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="50" customWidth="1"/>
+    <col min="18" max="19" width="45" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -153,3157 +206,3383 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>0C11108026419D776229</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>NON_ESEGUITO</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J2">
+      <c r="J2" s="2">
         <v>43.591353</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="2">
         <v>10.473372</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="2">
         <v>384.6</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="4">
         <v>0.385</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591353,10.473372</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>0D01C4A3D9419D77F4F8</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 ESEGUITO</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Eseguita)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>ESEGUITO</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>43.597359</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="2">
         <v>10.478268</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="2">
         <v>580.3</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="4">
         <v>0.58</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>Tratta stabilita con un walk-in in data 29/09/2026 e 03/10/2026. Si notano minitrincee, matasse di corrugati e birilli. Oltre a una serie di pozzetti Fibercop.</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.597359,10.478268</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>038A8E74E7419D783FA8</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>C [01] ARL</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>43.595685</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="2">
         <v>10.474887</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="3">
         <v>14.3</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione | Apparato supplementare | Tombini Telecom e TIM vicini</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.595685,10.474887</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>0D4F245AFD419D79C210</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>C [02] ARL</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J5">
+      <c r="J5" s="2">
         <v>43.591096</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="2">
         <v>10.475529</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="3">
         <v>25.8</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione | Apparato aggiuntivo | Tombino Telecom datato</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591096,10.475529</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>0F23EA90BA419D7FECB9</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>C [04] ARL</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J6">
+      <c r="J6" s="2">
         <v>43.588583</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="2">
         <v>10.473953</v>
       </c>
-      <c r="L6">
+      <c r="L6" s="3">
         <v>21.4</v>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
         <is>
           <t>Solo ARL</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.588583,10.473953</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>0F8841432F419D838E0B</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>C [9605] ARL</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J7">
+      <c r="J7" s="2">
         <v>43.588526</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="2">
         <v>10.472213</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="3">
         <v>23.0</v>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t>Solo ARL</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.588526,10.472213</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>030934D8B9419D824C48</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>C [9606] ARL</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J8">
+      <c r="J8" s="2">
         <v>43.58851</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="2">
         <v>10.47337</v>
       </c>
-      <c r="L8">
+      <c r="L8" s="3">
         <v>26.4</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.58851,10.47337</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>0C1639DB3D41C037B01F</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>C [07] ARL</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J9">
+      <c r="J9" s="2">
         <v>43.593381</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="2">
         <v>10.471502</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="3">
         <v>13.0</v>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.593381,10.471502</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>051EB54D5C419D7EA6D4</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>C [08] ARL</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J10">
+      <c r="J10" s="2">
         <v>43.587389</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="2">
         <v>10.476109</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="3">
         <v>47.0</v>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t>Solo ARL | NUMERO DA VERIFICARE IRL</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.587389,10.476109</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>06A6E2BD72419DA42506</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>V [01] ARL</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J11">
+      <c r="J11" s="2">
         <v>43.615979</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="2">
         <v>10.463939</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="3">
         <v>8.9</v>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t>Piccolo apparato e-distribuzione appeso allo SLAM</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.615979,10.463939</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>0698C7718E419DA0FA44</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>V [02] ARL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J12">
+      <c r="J12" s="2">
         <v>43.614158</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="2">
         <v>10.464706</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="3">
         <v>8.3</v>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione | Apparato aggiuntivo | Tombini TIM e INWIT</t>
         </is>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.614158,10.464706</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>0ECF9F5C0F419DA225A1</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>V [03] ARL</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J13">
+      <c r="J13" s="2">
         <v>43.611401</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="2">
         <v>10.462766</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="3">
         <v>7.2</v>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="R13" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.611401,10.462766</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>0305AC62A2419D9EC684</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>V [04] ARL</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J14">
+      <c r="J14" s="2">
         <v>43.611423</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="2">
         <v>10.467038</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="3">
         <v>9.4</v>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="Q14" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R14" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.611423,10.467038</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>0047495E12419D9FD2E4</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>V [05] ARL</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J15">
+      <c r="J15" s="2">
         <v>43.608954</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="2">
         <v>10.468205</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="3">
         <v>9.9</v>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="Q15" s="2" t="inlineStr">
         <is>
           <t>Solo ARL | NUOVO DAL 2025</t>
         </is>
       </c>
-      <c r="R15" t="inlineStr">
+      <c r="R15" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.608954,10.468205</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>0E749B0B68419D9E6D0F</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>V [06] ARL</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J16">
+      <c r="J16" s="2">
         <v>43.607712</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="2">
         <v>10.469103</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="3">
         <v>20.1</v>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="Q16" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R16" t="inlineStr">
+      <c r="R16" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.607712,10.469103</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>0EE4D73D73419DA346CF</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>V [07] ARL</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J17">
+      <c r="J17" s="2">
         <v>43.60849</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="2">
         <v>10.459436</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="3">
         <v>8.1</v>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R17" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.60849,10.459436</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>086A77D7C1419DA6C13B</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>V [08] ARL</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J18">
+      <c r="J18" s="2">
         <v>43.605143</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="2">
         <v>10.440451</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="3">
         <v>6.2</v>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="Q18" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R18" t="inlineStr">
+      <c r="R18" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.605143,10.440451</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>073CCE441A419DEDF933</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>S [28] ARLO</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>ARLO (Ottico FiberCop)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J19">
+      <c r="J19" s="2">
         <v>43.590687</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="2">
         <v>10.35622</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="3">
         <v>9.2</v>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R19" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.590687,10.35622</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>0B539CBC0B41A1D9DE66</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>S [02] ARL</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J20">
+      <c r="J20" s="2">
         <v>43.592438</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="2">
         <v>10.350568</v>
       </c>
-      <c r="L20">
+      <c r="L20" s="3">
         <v>2.5</v>
       </c>
-      <c r="Q20" t="inlineStr">
+      <c r="Q20" s="2" t="inlineStr">
         <is>
           <t>Con apparato aggiuntivo</t>
         </is>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R20" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.592438,10.350568</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>0263F1596941C03C8160</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>S [04] ARL</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J21">
+      <c r="J21" s="2">
         <v>43.589338</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="2">
         <v>10.353907</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="3">
         <v>5.4</v>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q21" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R21" t="inlineStr">
+      <c r="R21" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.589338,10.353907</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>08BC1C303941A1DD1397</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>S [05] ARL</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J22">
+      <c r="J22" s="2">
         <v>43.590359</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="2">
         <v>10.353377</v>
       </c>
-      <c r="L22">
+      <c r="L22" s="3">
         <v>12.5</v>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q22" s="2" t="inlineStr">
         <is>
           <t>Solo ARL</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr">
+      <c r="R22" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.590359,10.353377</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>0E5AD376F741A1E1369B</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>S [07] ARL</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J23">
+      <c r="J23" s="2">
         <v>43.589462</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="2">
         <v>10.349117</v>
       </c>
-      <c r="L23">
+      <c r="L23" s="3">
         <v>2.7</v>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" s="2" t="inlineStr">
         <is>
           <t>Solo ARL</t>
         </is>
       </c>
-      <c r="R23" t="inlineStr">
+      <c r="R23" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.589462,10.349117</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>0D98E9743941A1DA3CA8</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Coppie di corrugati scoperti</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Infrastruttura / Corrugati</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Altro</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J24">
+      <c r="J24" s="2">
         <v>43.591341</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="2">
         <v>10.350005</v>
       </c>
-      <c r="L24">
+      <c r="L24" s="3">
         <v>2.4</v>
       </c>
-      <c r="R24" t="inlineStr">
+      <c r="R24" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591341,10.350005</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>017CFF11F041A1FE2121</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>G [01] ARL</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Guasticce</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J25">
+      <c r="J25" s="2">
         <v>43.597713</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="2">
         <v>10.408314</v>
       </c>
-      <c r="L25">
+      <c r="L25" s="3">
         <v>4.3</v>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="Q25" s="2" t="inlineStr">
         <is>
           <t>Solo ARL | Tombini TIM vicini</t>
         </is>
       </c>
-      <c r="R25" t="inlineStr">
+      <c r="R25" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.597713,10.408314</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>0D6146352741A1FCE21E</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>G [02] ARL</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Guasticce</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J26">
+      <c r="J26" s="2">
         <v>43.597372</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="2">
         <v>10.405911</v>
       </c>
-      <c r="L26">
+      <c r="L26" s="3">
         <v>4.9</v>
       </c>
-      <c r="Q26" t="inlineStr">
+      <c r="Q26" s="2" t="inlineStr">
         <is>
           <t>Colonnina e-distribuzione</t>
         </is>
       </c>
-      <c r="R26" t="inlineStr">
+      <c r="R26" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.597372,10.405911</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>03D89618D341A1FAF659</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>G [0?] ARL</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Guasticce</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J27">
+      <c r="J27" s="2">
         <v>43.59665</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="2">
         <v>10.391757</v>
       </c>
-      <c r="L27">
+      <c r="L27" s="3">
         <v>2.8</v>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="Q27" s="2" t="inlineStr">
         <is>
           <t>Alimentazione e-distribuzione appesa allo SLAM | Da verificare numero IRL</t>
         </is>
       </c>
-      <c r="R27" t="inlineStr">
+      <c r="R27" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.59665,10.391757</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>01B27264D9419D7C94C9</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Centrale Comunale (Collesalvetti)</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Centrale Telecom (Sede OLT)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J28">
+      <c r="J28" s="2">
         <v>43.587841</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="2">
         <v>10.477201</v>
       </c>
-      <c r="L28">
+      <c r="L28" s="3">
         <v>47.5</v>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="Q28" s="2" t="inlineStr">
         <is>
           <t>XGS-PON (10 gigabit) | Tombini Telecom, TIM e Fastweb (quest'ultimo per allacciare Casa di Riposo Santa Caterina)</t>
         </is>
       </c>
-      <c r="R28" t="inlineStr">
+      <c r="R28" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.587841,10.477201</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>01700D6671419DAEA488</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Vicarello)</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Vicarello</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J29">
+      <c r="J29" s="2">
         <v>43.608339</v>
       </c>
-      <c r="K29">
+      <c r="K29" s="2">
         <v>10.471259</v>
       </c>
-      <c r="L29">
+      <c r="L29" s="3">
         <v>17.1</v>
       </c>
-      <c r="R29" t="inlineStr">
+      <c r="R29" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.608339,10.471259</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>05ACF8364E419DAFCD6E</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Guasticce)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Guasticce</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J30">
+      <c r="J30" s="2">
         <v>43.596228</v>
       </c>
-      <c r="K30">
+      <c r="K30" s="2">
         <v>10.406849</v>
       </c>
-      <c r="L30">
+      <c r="L30" s="3">
         <v>8.2</v>
       </c>
-      <c r="R30" t="inlineStr">
+      <c r="R30" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.596228,10.406849</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>0BCA63C363419DB26088</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Nugola)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Nugola</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J31">
+      <c r="J31" s="2">
         <v>43.577525</v>
       </c>
-      <c r="K31">
+      <c r="K31" s="2">
         <v>10.438356</v>
       </c>
-      <c r="L31">
+      <c r="L31" s="3">
         <v>67.0</v>
       </c>
-      <c r="R31" t="inlineStr">
+      <c r="R31" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.577525,10.438356</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>09ECE9F1E7419DB39FB6</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Parrana San Martino)</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Parrana San Martino</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J32">
+      <c r="J32" s="2">
         <v>43.538167</v>
       </c>
-      <c r="K32">
+      <c r="K32" s="2">
         <v>10.442333</v>
       </c>
-      <c r="L32">
+      <c r="L32" s="3">
         <v>0.0</v>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="Q32" s="2" t="inlineStr">
         <is>
           <t>Frazione di Parrana San Martino</t>
         </is>
       </c>
-      <c r="R32" t="inlineStr">
+      <c r="R32" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.538167,10.442333</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>057A74F77A419DB426D9</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Parrana San Giusto)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Parrana San Giusto</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J33">
+      <c r="J33" s="2">
         <v>43.528528</v>
       </c>
-      <c r="K33">
+      <c r="K33" s="2">
         <v>10.457333</v>
       </c>
-      <c r="L33">
+      <c r="L33" s="3">
         <v>0.0</v>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="Q33" s="2" t="inlineStr">
         <is>
           <t>Frazione di Parrana San Giusto</t>
         </is>
       </c>
-      <c r="R33" t="inlineStr">
+      <c r="R33" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.528528,10.457333</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>03B291C7F3419DB5DFC8</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione (Stagno)</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Centrale di Frazione</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J34">
+      <c r="J34" s="2">
         <v>43.586222</v>
       </c>
-      <c r="K34">
+      <c r="K34" s="2">
         <v>10.347222</v>
       </c>
-      <c r="L34">
+      <c r="L34" s="3">
         <v>0.0</v>
       </c>
-      <c r="R34" t="inlineStr">
+      <c r="R34" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.586222,10.347222</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>0F80C4A9C341A1D76E6B</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J35">
+      <c r="J35" s="2">
         <v>43.591686</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="2">
         <v>10.348608</v>
       </c>
-      <c r="M35">
+      <c r="M35" s="2">
         <v>1833.4</v>
       </c>
-      <c r="N35">
+      <c r="N35" s="4">
         <v>1.833</v>
       </c>
-      <c r="R35" t="inlineStr">
+      <c r="R35" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591686,10.348608</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>06D81465DD41A1D7D42C</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J36">
+      <c r="J36" s="2">
         <v>43.594286</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="2">
         <v>10.351331</v>
       </c>
-      <c r="M36">
+      <c r="M36" s="2">
         <v>346.9</v>
       </c>
-      <c r="N36">
+      <c r="N36" s="4">
         <v>0.347</v>
       </c>
-      <c r="R36" t="inlineStr">
+      <c r="R36" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.594286,10.351331</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>0C88D2EDB941A20C5424</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>INFRATEL</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Infrastruttura Infratel BUL</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Altro</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J37">
+      <c r="J37" s="2">
         <v>43.596264</v>
       </c>
-      <c r="K37">
+      <c r="K37" s="2">
         <v>10.406675</v>
       </c>
-      <c r="M37">
+      <c r="M37" s="2">
         <v>6533.3</v>
       </c>
-      <c r="N37">
+      <c r="N37" s="4">
         <v>6.533</v>
       </c>
-      <c r="Q37" t="inlineStr">
+      <c r="Q37" s="2" t="inlineStr">
         <is>
           <t>TORSFNUGOLANUOVA | Un percorso con un misto di palifica, cavidotto e mini trincea per rilegare in fibra ottica le centrali Fibercop usando il progetto del MISR 2014-2020</t>
         </is>
       </c>
-      <c r="R37" t="inlineStr">
+      <c r="R37" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.596264,10.406675</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>02442DD76E41BFC6C1C1</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>NON_ESEGUITO</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J38">
+      <c r="J38" s="2">
         <v>43.593705</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="2">
         <v>10.474944</v>
       </c>
-      <c r="M38">
+      <c r="M38" s="2">
         <v>96.5</v>
       </c>
-      <c r="N38">
+      <c r="N38" s="4">
         <v>0.097</v>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q38" s="2" t="inlineStr">
         <is>
           <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
-      <c r="R38" t="inlineStr">
+      <c r="R38" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.593705,10.474944</t>
         </is>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="S38" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>099D51459541BFC79191</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>NON_ESEGUITO</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J39">
+      <c r="J39" s="2">
         <v>43.592936</v>
       </c>
-      <c r="K39">
+      <c r="K39" s="2">
         <v>10.47365</v>
       </c>
-      <c r="M39">
+      <c r="M39" s="2">
         <v>513.7</v>
       </c>
-      <c r="N39">
+      <c r="N39" s="4">
         <v>0.514</v>
       </c>
-      <c r="Q39" t="inlineStr">
+      <c r="Q39" s="2" t="inlineStr">
         <is>
           <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr">
+      <c r="R39" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.592936,10.47365</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="S39" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>08DB97EDC341BFC840B3</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 ESEGUITO</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Eseguita)</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>ESEGUITO</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J40">
+      <c r="J40" s="2">
         <v>43.595583</v>
       </c>
-      <c r="K40">
+      <c r="K40" s="2">
         <v>10.474905</v>
       </c>
-      <c r="M40">
+      <c r="M40" s="2">
         <v>496.3</v>
       </c>
-      <c r="N40">
+      <c r="N40" s="4">
         <v>0.496</v>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q40" s="2" t="inlineStr">
         <is>
           <t>Tratta stabilita con un walk-in in data 29/09/2026 e 03/10/2026. Si notano minitrincee, matasse di corrugati e birilli. Oltre a una serie di pozzetti Fibercop.</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="R40" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.595583,10.474905</t>
         </is>
       </c>
-      <c r="S40" t="inlineStr">
+      <c r="S40" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>0B6DD449B041BFC99520</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>NON_ESEGUITO</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J41">
+      <c r="J41" s="2">
         <v>43.593354</v>
       </c>
-      <c r="K41">
+      <c r="K41" s="2">
         <v>10.477089</v>
       </c>
-      <c r="M41">
+      <c r="M41" s="2">
         <v>340.9</v>
       </c>
-      <c r="N41">
+      <c r="N41" s="4">
         <v>0.341</v>
       </c>
-      <c r="Q41" t="inlineStr">
+      <c r="Q41" s="2" t="inlineStr">
         <is>
           <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
-      <c r="R41" t="inlineStr">
+      <c r="R41" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.593354,10.477089</t>
         </is>
       </c>
-      <c r="S41" t="inlineStr">
+      <c r="S41" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>08927D586B41BFCD66AB</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Area Coperta Collesalvetti</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Area Coperta FTTH</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="J42">
+      <c r="J42" s="2">
         <v>43.597352</v>
       </c>
-      <c r="K42">
+      <c r="K42" s="2">
         <v>10.478314</v>
       </c>
-      <c r="O42">
+      <c r="O42" s="2">
         <v>205512.9</v>
       </c>
-      <c r="P42">
+      <c r="P42" s="4">
         <v>0.2055</v>
       </c>
-      <c r="R42" t="inlineStr">
+      <c r="R42" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.597352,10.478314</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>08A788CB5441BFCE4768</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Area NON Coperta Collesalvetti</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Area NON Coperta</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="J43">
+      <c r="J43" s="2">
         <v>43.591043</v>
       </c>
-      <c r="K43">
+      <c r="K43" s="2">
         <v>10.471834</v>
       </c>
-      <c r="O43">
+      <c r="O43" s="2">
         <v>455950.0</v>
       </c>
-      <c r="P43">
+      <c r="P43" s="4">
         <v>0.456</v>
       </c>
-      <c r="R43" t="inlineStr">
+      <c r="R43" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591043,10.471834</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>0F1AE3268141C0558FB7</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Tratto Scuole Connesse</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Tratta Scuole Connesse</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J44">
+      <c r="J44" s="2">
         <v>43.595701</v>
       </c>
-      <c r="K44">
+      <c r="K44" s="2">
         <v>10.474857</v>
       </c>
-      <c r="M44">
+      <c r="M44" s="2">
         <v>345.6</v>
       </c>
-      <c r="N44">
+      <c r="N44" s="4">
         <v>0.346</v>
       </c>
-      <c r="Q44" t="inlineStr">
+      <c r="Q44" s="2" t="inlineStr">
         <is>
           <t>Realizzato nel 2025-2026, una decina di pozzetti marchio Fibercop (logo nuovo). Collega ARL 01 a Scuole medie e la nuova struttura di asilo nido "I cubi". Hanno fatto delle mini-trincee</t>
         </is>
       </c>
-      <c r="R44" t="inlineStr">
+      <c r="R44" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.595701,10.474857</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>03A16F4CC141C0599BFE</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Tratto Sanità Connesse</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Tratta Sanità Connesse</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J45">
+      <c r="J45" s="2">
         <v>43.587826</v>
       </c>
-      <c r="K45">
+      <c r="K45" s="2">
         <v>10.477238</v>
       </c>
-      <c r="M45">
+      <c r="M45" s="2">
         <v>348.3</v>
       </c>
-      <c r="N45">
+      <c r="N45" s="4">
         <v>0.348</v>
       </c>
-      <c r="Q45" t="inlineStr">
+      <c r="Q45" s="2" t="inlineStr">
         <is>
           <t>Realizzato nel 2026. Scavo per conto di Fastweb che ha vinto il bando per connettere le strutture sanitarie nel comune. Pozzetti Fastweb e mini-trincee. Collega la centrale Fibercop a Casa di Riposo Santa Caterina e USL Collesalvetti.</t>
         </is>
       </c>
-      <c r="R45" t="inlineStr">
+      <c r="R45" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.587826,10.477238</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>0F2DA583D541C062FA84</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Area Coperta Stagno</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Area Coperta FTTH</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="J46">
+      <c r="J46" s="2">
         <v>43.591561</v>
       </c>
-      <c r="K46">
+      <c r="K46" s="2">
         <v>10.348533</v>
       </c>
-      <c r="O46">
+      <c r="O46" s="2">
         <v>371709.9</v>
       </c>
-      <c r="P46">
+      <c r="P46" s="4">
         <v>0.3717</v>
       </c>
-      <c r="R46" t="inlineStr">
+      <c r="R46" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591561,10.348533</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>07BBF594BC41C065D329</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Area NON Coperta Stagno</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Area NON Coperta</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Polygon</t>
         </is>
       </c>
-      <c r="J47">
+      <c r="J47" s="2">
         <v>43.589887</v>
       </c>
-      <c r="K47">
+      <c r="K47" s="2">
         <v>10.347674</v>
       </c>
-      <c r="O47">
+      <c r="O47" s="2">
         <v>91283.7</v>
       </c>
-      <c r="P47">
+      <c r="P47" s="4">
         <v>0.0913</v>
       </c>
-      <c r="R47" t="inlineStr">
+      <c r="R47" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.589887,10.347674</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>0AD5AAF68741C10071CC</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>PROGRAMMATO</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>2026-09-21 -&gt; 2026-10-16</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 95 del 10/09/2026 (Reg. Gen. 102)</t>
         </is>
       </c>
-      <c r="J48">
+      <c r="J48" s="2">
         <v>43.590227</v>
       </c>
-      <c r="K48">
+      <c r="K48" s="2">
         <v>10.353891</v>
       </c>
-      <c r="M48">
+      <c r="M48" s="2">
         <v>792.4</v>
       </c>
-      <c r="N48">
+      <c r="N48" s="4">
         <v>0.792</v>
       </c>
-      <c r="Q48" t="inlineStr">
+      <c r="Q48" s="2" t="inlineStr">
         <is>
           <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
-      <c r="R48" t="inlineStr">
+      <c r="R48" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.590227,10.353891</t>
         </is>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S48" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_102_2026_stagno_cantiere2.pdf</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>04D8D17C9141C10125EB</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>PROGRAMMATO</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>2026-09-21 -&gt; 2026-10-16</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 95 del 10/09/2026 (Reg. Gen. 102)</t>
         </is>
       </c>
-      <c r="J49">
+      <c r="J49" s="2">
         <v>43.590159</v>
       </c>
-      <c r="K49">
+      <c r="K49" s="2">
         <v>10.353883</v>
       </c>
-      <c r="M49">
+      <c r="M49" s="2">
         <v>360.5</v>
       </c>
-      <c r="N49">
+      <c r="N49" s="4">
         <v>0.36</v>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="Q49" s="2" t="inlineStr">
         <is>
           <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
-      <c r="R49" t="inlineStr">
+      <c r="R49" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.590159,10.353883</t>
         </is>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="S49" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_102_2026_stagno_cantiere2.pdf</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>01393CA83D41C1030753</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Cantiere 2 (05/10-17/10)</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>PROGRAMMATO</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>2026-09-21 -&gt; 2026-10-16</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>Via Otto Marzo, Via Romita, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 95 del 10/09/2026 (Reg. Gen. 102)</t>
         </is>
       </c>
-      <c r="J50">
+      <c r="J50" s="2">
         <v>43.588516</v>
       </c>
-      <c r="K50">
+      <c r="K50" s="2">
         <v>10.353942</v>
       </c>
-      <c r="M50">
+      <c r="M50" s="2">
         <v>277.9</v>
       </c>
-      <c r="N50">
+      <c r="N50" s="4">
         <v>0.278</v>
       </c>
-      <c r="Q50" t="inlineStr">
+      <c r="Q50" s="2" t="inlineStr">
         <is>
           <t>Slittato... vecchia data 21/09-16/10</t>
         </is>
       </c>
-      <c r="R50" t="inlineStr">
+      <c r="R50" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.588516,10.353942</t>
         </is>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="S50" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_102_2026_stagno_cantiere2.pdf</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>05C7B1F97841C1CA147C</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>Opera sulla Backbone di 07/2026</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Dorsale / Backbone Fibra</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J51">
+      <c r="J51" s="2">
         <v>43.571782</v>
       </c>
-      <c r="K51">
+      <c r="K51" s="2">
         <v>10.369152</v>
       </c>
-      <c r="M51">
+      <c r="M51" s="2">
         <v>519.2</v>
       </c>
-      <c r="N51">
+      <c r="N51" s="4">
         <v>0.519</v>
       </c>
-      <c r="Q51" t="inlineStr">
+      <c r="Q51" s="2" t="inlineStr">
         <is>
           <t>Opera di Fibercop su una tratta di backbone in fibra che va verso est quindi presumibilmente verso Collesalvetti. Ordinanza allegata...</t>
         </is>
       </c>
-      <c r="R51" t="inlineStr">
+      <c r="R51" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.571782,10.369152</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>05B932036B41C1D8F728</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>INFRATEL</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Infrastruttura Infratel BUL</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Altro</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J52">
+      <c r="J52" s="2">
         <v>43.538194</v>
       </c>
-      <c r="K52">
+      <c r="K52" s="2">
         <v>10.442316</v>
       </c>
-      <c r="M52">
+      <c r="M52" s="2">
         <v>3462.3</v>
       </c>
-      <c r="N52">
+      <c r="N52" s="4">
         <v>3.462</v>
       </c>
-      <c r="Q52" t="inlineStr">
+      <c r="Q52" s="2" t="inlineStr">
         <is>
           <t>Seconda ed ultima tratta di INFRATEL per rilegare le centrali di Parrana San Martino e Parrana San Giusto in fibra ottica. Prevalentemente in palifica (specialmente a nord-ovest)</t>
         </is>
       </c>
-      <c r="R52" t="inlineStr">
+      <c r="R52" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.538194,10.442316</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>0A2895209441C56CED8C</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>S [27] ARLO</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>ARLO (Ottico FiberCop)</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J53">
+      <c r="J53" s="2">
         <v>43.592688</v>
       </c>
-      <c r="K53">
+      <c r="K53" s="2">
         <v>10.350454</v>
       </c>
-      <c r="L53">
+      <c r="L53" s="3">
         <v>2.5</v>
       </c>
-      <c r="R53" t="inlineStr">
+      <c r="R53" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.592688,10.350454</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>06D2B51C4A41C5796F90</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>S [03] ARL</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>ARL (Rame)</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J54">
+      <c r="J54" s="2">
         <v>43.589284</v>
       </c>
-      <c r="K54">
+      <c r="K54" s="2">
         <v>10.355304</v>
       </c>
-      <c r="L54">
+      <c r="L54" s="3">
         <v>9.0</v>
       </c>
-      <c r="Q54" t="inlineStr">
+      <c r="Q54" s="2" t="inlineStr">
         <is>
           <t>Con apparato aggiuntivo</t>
         </is>
       </c>
-      <c r="R54" t="inlineStr">
+      <c r="R54" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.589284,10.355304</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>087416D75C41C59E4800</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J55">
+      <c r="J55" s="2">
         <v>43.59306</v>
       </c>
-      <c r="K55">
+      <c r="K55" s="2">
         <v>10.349492</v>
       </c>
-      <c r="M55">
+      <c r="M55" s="2">
         <v>250.1</v>
       </c>
-      <c r="N55">
+      <c r="N55" s="4">
         <v>0.25</v>
       </c>
-      <c r="R55" t="inlineStr">
+      <c r="R55" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.59306,10.349492</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>023213B9C541C59EFAE8</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J56">
+      <c r="J56" s="2">
         <v>43.592858</v>
       </c>
-      <c r="K56">
+      <c r="K56" s="2">
         <v>10.350051</v>
       </c>
-      <c r="M56">
+      <c r="M56" s="2">
         <v>119.4</v>
       </c>
-      <c r="N56">
+      <c r="N56" s="4">
         <v>0.119</v>
       </c>
-      <c r="R56" t="inlineStr">
+      <c r="R56" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.592858,10.350051</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>03B96D8A3141C59F56F7</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J57">
+      <c r="J57" s="2">
         <v>43.591477</v>
       </c>
-      <c r="K57">
+      <c r="K57" s="2">
         <v>10.349452</v>
       </c>
-      <c r="M57">
+      <c r="M57" s="2">
         <v>149.9</v>
       </c>
-      <c r="N57">
+      <c r="N57" s="4">
         <v>0.15</v>
       </c>
-      <c r="R57" t="inlineStr">
+      <c r="R57" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.591477,10.349452</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>0AB38499FF41C59FB9EC</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Tratta Stagno (Maggio 2026-Giugno 2026)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Tratta Fibra Posa</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="J58">
+      <c r="J58" s="2">
         <v>43.59114</v>
       </c>
-      <c r="K58">
+      <c r="K58" s="2">
         <v>10.350885</v>
       </c>
-      <c r="M58">
+      <c r="M58" s="2">
         <v>308.2</v>
       </c>
-      <c r="N58">
+      <c r="N58" s="4">
         <v>0.308</v>
       </c>
-      <c r="R58" t="inlineStr">
+      <c r="R58" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.59114,10.350885</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>04A0FAC1A941E16312D8</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Centrale Feeder (Livorno Nord)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Centrale Feeder (Interconnessione Esterna)</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Altro</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Point</t>
         </is>
       </c>
-      <c r="J59">
+      <c r="J59" s="2">
         <v>43.549556</v>
       </c>
-      <c r="K59">
+      <c r="K59" s="2">
         <v>10.310667</v>
       </c>
-      <c r="L59">
+      <c r="L59" s="3">
         <v>0.0</v>
       </c>
-      <c r="Q59" t="inlineStr">
+      <c r="Q59" s="2" t="inlineStr">
         <is>
           <t>Grande centrale Fibercop che funge da "feeder" alla centrale comunale di Collesalvetti</t>
         </is>
       </c>
-      <c r="R59" t="inlineStr">
+      <c r="R59" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.549556,10.310667</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>0DE7916F26423746716E</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Cantiere 1 NON ESEGUITO</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Cantiere FTTH (Tratta Non Eseguita)</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>Collesalvetti</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>NON_ESEGUITO</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 -&gt; 2026-10-02</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>Via Nenni, Via Roma (rotatoria Via Nenni), Via del Valico a Pisa, Via di Cerretello</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>Ordinanza P.M. n. 88 del 02/09/2026 (Reg. Gen. 95)</t>
         </is>
       </c>
-      <c r="J60">
+      <c r="J60" s="2">
         <v>43.595608</v>
       </c>
-      <c r="K60">
+      <c r="K60" s="2">
         <v>10.474975</v>
       </c>
-      <c r="M60">
+      <c r="M60" s="2">
         <v>182.8</v>
       </c>
-      <c r="N60">
+      <c r="N60" s="4">
         <v>0.183</v>
       </c>
-      <c r="Q60" t="inlineStr">
+      <c r="Q60" s="2" t="inlineStr">
         <is>
           <t>Si notano solamente dei segni blu (oltre ai soliti colori), che indicano Fibercop , sull'asfalto</t>
         </is>
       </c>
-      <c r="R60" t="inlineStr">
+      <c r="R60" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.595608,10.474975</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr">
+      <c r="S60" s="2" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_95_2026_collesalvetti_cantiere1.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>0A173E317742376CD0E8</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>Cantiere 3 (19/10-23/10)</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>Cantiere Fibra Ottica</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>DA COLLEGARE A ORDINANZA</t>
         </is>
       </c>
-      <c r="J61">
+      <c r="J61" s="2">
         <v>43.581537</v>
       </c>
-      <c r="K61">
+      <c r="K61" s="2">
         <v>10.350735</v>
       </c>
-      <c r="M61">
+      <c r="M61" s="2">
         <v>172.7</v>
       </c>
-      <c r="N61">
+      <c r="N61" s="4">
         <v>0.173</v>
       </c>
-      <c r="R61" t="inlineStr">
+      <c r="R61" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.581537,10.350735</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>0EB8D0BA5142376E2D37</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Cantiere 3 (19/10-23/10)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Cantiere Fibra Ottica</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>DA COLLEGARE A ORDINANZA</t>
         </is>
       </c>
-      <c r="J62">
+      <c r="J62" s="2">
         <v>43.58171</v>
       </c>
-      <c r="K62">
+      <c r="K62" s="2">
         <v>10.343732</v>
       </c>
-      <c r="M62">
+      <c r="M62" s="2">
         <v>627.5</v>
       </c>
-      <c r="N62">
+      <c r="N62" s="4">
         <v>0.627</v>
       </c>
-      <c r="R62" t="inlineStr">
+      <c r="R62" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.58171,10.343732</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>07624940EF4237721F0B</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Cantiere 3 (19/10-23/10)</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>Cantiere Fibra Ottica</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>DA COLLEGARE A ORDINANZA</t>
         </is>
       </c>
-      <c r="J63">
+      <c r="J63" s="2">
         <v>43.581465</v>
       </c>
-      <c r="K63">
+      <c r="K63" s="2">
         <v>10.348597</v>
       </c>
-      <c r="M63">
+      <c r="M63" s="2">
         <v>2507.4</v>
       </c>
-      <c r="N63">
+      <c r="N63" s="4">
         <v>2.507</v>
       </c>
-      <c r="Q63" t="inlineStr">
+      <c r="Q63" s="2" t="inlineStr">
         <is>
           <t>Improbabile che il cantiere arrivi fino a queste zone, ma fino al 24 ottobre circa terrò sulla mappa tutta Via Aiaccia. Curioso che però questa tratta arriva davanti alla tratta color viola "Opera sulla Backbone di 07/26"... analisi di questa informazione è necessaria.</t>
         </is>
       </c>
-      <c r="R63" t="inlineStr">
+      <c r="R63" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.581465,10.348597</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>0C884334EF423778B430</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Cantiere 3 (19/10-23/10)</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Cantiere Fibra Ottica</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Stagno</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>LineString</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>DA COLLEGARE A ORDINANZA</t>
         </is>
       </c>
-      <c r="J64">
+      <c r="J64" s="2">
         <v>43.58522</v>
       </c>
-      <c r="K64">
+      <c r="K64" s="2">
         <v>10.353831</v>
       </c>
-      <c r="M64">
+      <c r="M64" s="2">
         <v>167.7</v>
       </c>
-      <c r="N64">
+      <c r="N64" s="4">
         <v>0.168</v>
       </c>
-      <c r="R64" t="inlineStr">
+      <c r="R64" s="2" t="inlineStr">
         <is>
           <t>https://www.google.com/maps?q=43.58522,10.353831</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:S64"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="45" customWidth="1"/>
+    <col min="2" max="2" width="75" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>METADATI ESPORTAZIONE GEOFIBRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Progetto</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>GeoFibra Collesalvetti - Osservatorio Civico FTTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Comune</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Collesalvetti (LI), Toscana, Italia</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Rilievo sorgente</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Snapshot 3 (2026-10-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Sorgente dati KML</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>data/snapshots/rilievo_snapshot3.kml</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Data generazione dataset</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>CONTEGGI GEOSPAZIALI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Totale feature rilevate</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Elementi puntiformi (Point)</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Tratte lineari (LineString)</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Aree poligonali (Polygon)</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Estensione totale rete (km)</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>21.716</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>CONTEGGI APPARATI (Metodologia V1.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Armadi comunali (ARL + ARLO)</t>
+        </is>
+      </c>
+      <c r="B16" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Centrali comunali (Telecom Sede OLT + Frazione)</t>
+        </is>
+      </c>
+      <c r="B17" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Totale apparati nel territorio comunale</t>
+        </is>
+      </c>
+      <c r="B18" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Apparati di raccordo esterno (Feeder)</t>
+        </is>
+      </c>
+      <c r="B19" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>NOTE LEGALI E METODOLOGICHE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Avvertenza</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>I dati derivano da rilievi civici sul campo e ordinanze comunali di viabilita'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Natura del dato</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Non costituiscono dato ufficiale di copertura degli operatori TLC (FiberCop / Open Fiber / Infratel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Licenza e consultazione</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Progetto open data / civico: consultabile liberamente.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(arlo): correggi censimento ARLO di Stagno a 3 nodi effettivi (S [27], S [28], S [])
</commit_message>
<xml_diff>
--- a/data/rete_ftth_collesalvetti.xlsx
+++ b/data/rete_ftth_collesalvetti.xlsx
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>S [] ARLO (Futuro ARLO 04 - 6° nodo Stagno)</t>
+          <t>S [] ARLO (Senza etichetta - Affiancato ad ARL 04)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Armadio ottico FiberCop posato in affiancamento al rame S [04] ARL ([10.353902, 43.589311]) su Via Romita / angolo Via XXV Aprile. 6° ARLO individuato nell'ultimo walk-in dell'11/10/2026. In zona 6 pozzetti in fase di getto/chiusura finale nell'area del Cantiere 2. Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
+          <t>Armadio ottico FiberCop posato in affiancamento al rame S [04] ARL ([10.353902, 43.589311]) su Via Romita / angolo Via XXV Aprile (privo di etichetta numerica, futuro ARLO 04 - 3° ARLO censito a Stagno). Rilevato nel walk-in dell'11/10/2026. In zona 6 pozzetti in fase di getto/chiusura finale nell'area del Cantiere 2. Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -4670,204 +4670,6 @@
       <c r="U69" t="inlineStr">
         <is>
           <t>ordinanze/ordinanza_102_2026_stagno_cantiere2.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>pm_68</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>S [05] ARLO</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>ARLO (Ottico FiberCop)</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>Stagno</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>FiberCop</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Infrastrutturati / In fase di cablaggio e predisposizione secondaria</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="L70">
-        <v>43.590365</v>
-      </c>
-      <c r="M70">
-        <v>10.35336</v>
-      </c>
-      <c r="N70">
-        <v>12.5</v>
-      </c>
-      <c r="S70" t="inlineStr">
-        <is>
-          <t>Armadio ottico FiberCop S [05] ARLO (Via De Gasperi / Via Romita nord, affiancato a S [05] ARL). | Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
-        </is>
-      </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps?q=43.590365,10.35336</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>pm_69</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>S [06] ARLO</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>ARLO (Ottico FiberCop)</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Stagno</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>FiberCop</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Infrastrutturati / In fase di cablaggio e predisposizione secondaria</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
-        </is>
-      </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="L71">
-        <v>43.591025</v>
-      </c>
-      <c r="M71">
-        <v>10.349825</v>
-      </c>
-      <c r="N71">
-        <v>2.7</v>
-      </c>
-      <c r="S71" t="inlineStr">
-        <is>
-          <t>Armadio ottico FiberCop S [06] ARLO (Via Machiavelli / Via 8 Marzo, affiancato a S [06] ARL). | Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
-        </is>
-      </c>
-      <c r="T71" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps?q=43.591025,10.349825</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>pm_70</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>S [07] ARLO</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>ARLO (Ottico FiberCop)</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Stagno</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>FiberCop</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Point</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Infrastrutturati / In fase di cablaggio e predisposizione secondaria</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
-        <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
-        </is>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>2026-10-11</t>
-        </is>
-      </c>
-      <c r="L72">
-        <v>43.58947</v>
-      </c>
-      <c r="M72">
-        <v>10.349105</v>
-      </c>
-      <c r="N72">
-        <v>2.7</v>
-      </c>
-      <c r="S72" t="inlineStr">
-        <is>
-          <t>Armadio ottico FiberCop S [07] ARLO (Via Guerrazzi sud, affiancato a S [07] ARL). | Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
-        </is>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps?q=43.58947,10.349105</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(snapshot5): integra rilievi Snapshot 5, Cantiere 4, ordinanze al 16/10/2026 e rebranding Geo Fibra
- Integrazione Snapshot 5 KML (71 feature, 23.840 km totali)
- Inclusione Cantiere 4 a Stagno (Ord. 110/2026, 3 nuove tratte per 2,062 km)
- Aggiornamento poligoni copertura Stagno (espansione a 71.64 ha, perimetro non coperto a 4.46 ha)
- Recepimento ordinanze 16/10/2026: proroga Cantiere 2 (Ord. 111) e ripristino Via Rosselli (Ord. 112)
- Evidenziazione nel Tracker dei 3 cantieri concomitanti dal 19/10
- Rebranding completo dell'osservatorio in Geo Fibra e aggiornamento export
- Allineamento test suite (21/21 OK) e documentazione
</commit_message>
<xml_diff>
--- a/data/rete_ftth_collesalvetti.xlsx
+++ b/data/rete_ftth_collesalvetti.xlsx
@@ -390,7 +390,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Primo armadio ottico del capoluogo (C [] ARLO, futuro ARLO 01), situato nell'aiuola/marciapiede della rotatoria tra Via Roma, Via Nenni e Via Piero Ciampi. Plinto gettato, cabinet montato, 4 pozzetti di smistamento FiberCop posati a corona della rotatoria e raccordati a cavidotti TIM preesistenti. Stato: Installato (Opere civili completate - In attesa di soffiaggio fibra/PTE).</t>
+          <t>Primo ARLO della città di Collesalvetti. Posato in una finestra di tempo dal 04/10 al 10/10. Non ha ancora nessuna etichetta per individuarne il numero</t>
         </is>
       </c>
       <c r="R4" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Armadio ottico FiberCop S [27] ARLO. | Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
+          <t>Armadio ottico FiberCop S [27] ARLO a Stagno. Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
         </is>
       </c>
       <c r="R20" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>Armadio ottico FiberCop S [28] ARLO. | Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
+          <t>Armadio ottico FiberCop S [28] ARLO a Stagno. Stato: Infrastrutturati / In fase di cablaggio e predisposizione secondaria.</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
@@ -2636,10 +2636,15 @@
         <v>10.348533</v>
       </c>
       <c r="O51" s="2">
-        <v>371709.9</v>
+        <v>716388.3</v>
       </c>
       <c r="P51" s="4">
-        <v>0.3717</v>
+        <v>0.7164</v>
+      </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>Area Coperta Stagno: estesa verso sud e ovest per includere il comparto di Cantiere 3 e Cantiere 4 (Snapshot 5 - 17/10/2026).</t>
+        </is>
       </c>
       <c r="R51" s="2" t="inlineStr">
         <is>
@@ -2650,7 +2655,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>07BBF594BC41C065D329</t>
+          <t>095490C3EE4270E4B838</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2674,20 +2679,25 @@
         </is>
       </c>
       <c r="J52" s="2">
-        <v>43.589887</v>
+        <v>43.586258</v>
       </c>
       <c r="K52" s="2">
-        <v>10.347674</v>
+        <v>10.355003</v>
       </c>
       <c r="O52" s="2">
-        <v>91283.7</v>
+        <v>44638.2</v>
       </c>
       <c r="P52" s="4">
-        <v>0.0913</v>
+        <v>0.0446</v>
+      </c>
+      <c r="Q52" s="2" t="inlineStr">
+        <is>
+          <t>Area NON Coperta Stagno: ridotta a stretta fascia orientale (10.3547 - 10.3576, Snapshot 5 - 17/10/2026).</t>
+        </is>
       </c>
       <c r="R52" s="2" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps?q=43.589887,10.347674</t>
+          <t>https://www.google.com/maps?q=43.586258,10.355003</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2734,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 -&gt; 2026-10-17</t>
+          <t>2026-09-21 -&gt; 2026-10-23</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2734,7 +2744,7 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
+          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026) + Proroga Ord. n. 111 del 16/10/2026</t>
         </is>
       </c>
       <c r="J53" s="2">
@@ -2751,7 +2761,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>Cantiere 2 Stagno (Ord. 104/2026). Finestra: 05/10/2026 - 17/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale).</t>
+          <t>Cantiere 2 Stagno (Ord. 104/2026 + Proroga Ord. 111 del 16/10/2026). Nuova scadenza: 23/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale attorno ad ARLO).</t>
         </is>
       </c>
       <c r="R53" s="2" t="inlineStr">
@@ -2798,7 +2808,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 -&gt; 2026-10-17</t>
+          <t>2026-09-21 -&gt; 2026-10-23</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -2808,7 +2818,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
+          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026) + Proroga Ord. n. 111 del 16/10/2026</t>
         </is>
       </c>
       <c r="J54" s="2">
@@ -2825,7 +2835,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>Cantiere 2 Stagno (Ord. 104/2026). Finestra: 05/10/2026 - 17/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale).</t>
+          <t>Cantiere 2 Stagno (Ord. 104/2026 + Proroga Ord. 111 del 16/10/2026). Nuova scadenza: 23/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale attorno ad ARLO).</t>
         </is>
       </c>
       <c r="R54" s="2" t="inlineStr">
@@ -2872,7 +2882,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 -&gt; 2026-10-17</t>
+          <t>2026-09-21 -&gt; 2026-10-23</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2882,7 +2892,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
+          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026) + Proroga Ord. n. 111 del 16/10/2026</t>
         </is>
       </c>
       <c r="J55" s="2">
@@ -2899,7 +2909,7 @@
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>Cantiere 2 Stagno (Ord. 104/2026). Finestra: 05/10/2026 - 17/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale).</t>
+          <t>Cantiere 2 Stagno (Ord. 104/2026 + Proroga Ord. 111 del 16/10/2026). Nuova scadenza: 23/10/2026. Vie: Via Romita sud, Via De Gasperi, Via Machiavelli, Via XXV Aprile, Piazza Di Vittorio, Via Don Verità, Via 8 Marzo. Stato: In completamento (Posa condotte completata, 6 pozzetti in fase di getto/chiusura finale attorno ad ARLO).</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -3710,7 +3720,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21 -&gt; 2026-10-17</t>
+          <t>2026-09-21 -&gt; 2026-10-23</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3720,7 +3730,7 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026)</t>
+          <t>Ordinanza P.M. n. 95/2026 (Reg. Gen. 102/104/2026) + Proroga Ord. n. 111 del 16/10/2026</t>
         </is>
       </c>
       <c r="J69" s="2">
@@ -3737,7 +3747,7 @@
       </c>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t>Tratta completata Cantiere 2 Stagno (Via Romita sud / Via XXV Aprile, 292,9 m). Posa condotte ultimata al walk-in 11/10/2026. Ord. 104/2026.</t>
+          <t>Tratta completata Cantiere 2 Stagno (Via Romita sud / Via XXV Aprile, 292,9 m). Posa condotte ultimata al walk-in 11/10/2026. Ord. 104/2026 prorogata con Ord. 111/2026.</t>
         </is>
       </c>
       <c r="R69" s="2" t="inlineStr">
@@ -3751,8 +3761,230 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>0766EAF8C74270D6924F</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 (26/10 - 20/11)</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 -&gt; 2026-11-20</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>Ordinanza P.M. n. 110/2026 (Autorizzazione Tecnica n. 26/2026)</t>
+        </is>
+      </c>
+      <c r="J70" s="2">
+        <v>43.591353</v>
+      </c>
+      <c r="K70" s="2">
+        <v>10.349463</v>
+      </c>
+      <c r="M70" s="2">
+        <v>1190.1</v>
+      </c>
+      <c r="N70" s="4">
+        <v>1.19</v>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 Stagno (Ordinanza PM n. 110/2026, Autorizzazione Tecnica n. 26/2026). Finestra: 26/10/2026 - 20/11/2026. Vie: Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer. Stato: Pianificato.</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.591353,10.349463</t>
+        </is>
+      </c>
+      <c r="S70" s="2" t="inlineStr">
+        <is>
+          <t>ordinanze/ordinanza_110_2026_stagno_cantiere4.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>012D8BFFFE4270DC0BCC</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 (26/10 - 20/11)</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 -&gt; 2026-11-20</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Ordinanza P.M. n. 110/2026 (Autorizzazione Tecnica n. 26/2026)</t>
+        </is>
+      </c>
+      <c r="J71" s="2">
+        <v>43.588977</v>
+      </c>
+      <c r="K71" s="2">
+        <v>10.347283</v>
+      </c>
+      <c r="M71" s="2">
+        <v>757.3</v>
+      </c>
+      <c r="N71" s="4">
+        <v>0.757</v>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 Stagno (Ordinanza PM n. 110/2026, Autorizzazione Tecnica n. 26/2026). Finestra: 26/10/2026 - 20/11/2026. Vie: Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer. Stato: Pianificato.</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.588977,10.347283</t>
+        </is>
+      </c>
+      <c r="S71" s="2" t="inlineStr">
+        <is>
+          <t>ordinanze/ordinanza_110_2026_stagno_cantiere4.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>0B718B800C4270DCE3E0</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 (26/10 - 20/11)</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere FTTH (Nuova Ordinanza Programmata)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Stagno</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>LineString</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 -&gt; 2026-11-20</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>Ordinanza P.M. n. 110/2026 (Autorizzazione Tecnica n. 26/2026)</t>
+        </is>
+      </c>
+      <c r="J72" s="2">
+        <v>43.587091</v>
+      </c>
+      <c r="K72" s="2">
+        <v>10.346453</v>
+      </c>
+      <c r="M72" s="2">
+        <v>115.3</v>
+      </c>
+      <c r="N72" s="4">
+        <v>0.115</v>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>Cantiere 4 Stagno (Ordinanza PM n. 110/2026, Autorizzazione Tecnica n. 26/2026). Finestra: 26/10/2026 - 20/11/2026. Vie: Via Marx, Via Curiel (lato sud), Via Gobetti, Via Don Verità, Via F.lli Cervi, Via La Malfa, Via Verga, Via Berlinguer. Stato: Pianificato.</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps?q=43.587091,10.346453</t>
+        </is>
+      </c>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>ordinanze/ordinanza_110_2026_stagno_cantiere4.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S69"/>
+  <autoFilter ref="A1:S72"/>
 </worksheet>
 </file>
 
@@ -3802,7 +4034,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Snapshot 4 (2026-10-11)</t>
+          <t>Snapshot 5 (2026-10-17)</t>
         </is>
       </c>
     </row>
@@ -3844,7 +4076,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -3864,7 +4096,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -3884,7 +4116,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>21.778</v>
+        <v>23.84</v>
       </c>
     </row>
     <row r="15">

</xml_diff>